<commit_message>
Add a college code alongside name, location and address
Colleges gain an optional short code (VTU-style "1RV", or any internal
reference). It is uppercased by the same setter as the name so the list reads
consistently, and it is explicitly not the identity — a college is still
identified by its name, so adding codes to an existing list cannot create
duplicates.

The code is captured in the single-add form, carried through the bulk importer
from either a "College Code" column or the second position when pasting, and
shown wherever a college is offered: as a badge in the admin list, beside the
name in the builder's picker, and as "NAME (CODE)" on the public form. It is
searchable in both the admin list and the picker.

The bundled template workbook gains the column and real VTU codes for its
twenty sample colleges.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/College-List-Template.xlsx
+++ b/docs/College-List-Template.xlsx
@@ -12,11 +12,14 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="85">
   <si>
     <t>College Name</t>
   </si>
   <si>
+    <t>College Code</t>
+  </si>
+  <si>
     <t>Location</t>
   </si>
   <si>
@@ -26,6 +29,9 @@
     <t>RV College of Engineering</t>
   </si>
   <si>
+    <t>1RV</t>
+  </si>
+  <si>
     <t>Bengaluru</t>
   </si>
   <si>
@@ -35,84 +41,126 @@
     <t>BMS College of Engineering</t>
   </si>
   <si>
+    <t>1BM</t>
+  </si>
+  <si>
     <t>Bull Temple Road, Basavanagudi, Bengaluru 560019</t>
   </si>
   <si>
     <t>PES University</t>
   </si>
   <si>
+    <t>1PE</t>
+  </si>
+  <si>
     <t>100 Feet Ring Road, BSK III Stage, Bengaluru 560085</t>
   </si>
   <si>
     <t>MS Ramaiah Institute of Technology</t>
   </si>
   <si>
+    <t>1MS</t>
+  </si>
+  <si>
     <t>MSR Nagar, MSRIT Post, Bengaluru 560054</t>
   </si>
   <si>
     <t>Bangalore Institute of Technology</t>
   </si>
   <si>
+    <t>1BI</t>
+  </si>
+  <si>
     <t>KR Road, VV Puram, Bengaluru 560004</t>
   </si>
   <si>
     <t>Dayananda Sagar College of Engineering</t>
   </si>
   <si>
+    <t>1DS</t>
+  </si>
+  <si>
     <t>Shavige Malleshwara Hills, Kumaraswamy Layout, Bengaluru 560078</t>
   </si>
   <si>
     <t>New Horizon College of Engineering</t>
   </si>
   <si>
+    <t>1NH</t>
+  </si>
+  <si>
     <t>Ring Road, Bellandur Post, Bengaluru 560103</t>
   </si>
   <si>
     <t>Acharya Institute of Technology</t>
   </si>
   <si>
+    <t>1AY</t>
+  </si>
+  <si>
     <t>Soldevanahalli, Hesaraghatta Road, Bengaluru 560107</t>
   </si>
   <si>
     <t>Sir M Visvesvaraya Institute of Technology</t>
   </si>
   <si>
+    <t>1MV</t>
+  </si>
+  <si>
     <t>Hunasamaranahalli, Yelahanka, Bengaluru 562157</t>
   </si>
   <si>
     <t>T John Institute of Technology</t>
   </si>
   <si>
+    <t>1TJ</t>
+  </si>
+  <si>
     <t>Gottigere, Bannerghatta Road, Bengaluru 560083</t>
   </si>
   <si>
     <t>Nitte Meenakshi Institute of Technology</t>
   </si>
   <si>
+    <t>1NT</t>
+  </si>
+  <si>
     <t>Govindapura, Yelahanka, Bengaluru 560064</t>
   </si>
   <si>
     <t>Sambhram Institute of Technology</t>
   </si>
   <si>
+    <t>1SB</t>
+  </si>
+  <si>
     <t>MS Palya, Jalahalli East, Bengaluru 560097</t>
   </si>
   <si>
     <t>CMR Institute of Technology</t>
   </si>
   <si>
+    <t>1CR</t>
+  </si>
+  <si>
     <t>AECS Layout, ITPL Main Road, Bengaluru 560037</t>
   </si>
   <si>
     <t>Global Academy of Technology</t>
   </si>
   <si>
+    <t>1GA</t>
+  </si>
+  <si>
     <t>Rajarajeshwari Nagar, Bengaluru 560098</t>
   </si>
   <si>
     <t>Siddaganga Institute of Technology</t>
   </si>
   <si>
+    <t>1SI</t>
+  </si>
+  <si>
     <t>Tumakuru</t>
   </si>
   <si>
@@ -122,6 +170,9 @@
     <t>PES Institute of Technology and Management</t>
   </si>
   <si>
+    <t>4PS</t>
+  </si>
+  <si>
     <t>Shivamogga</t>
   </si>
   <si>
@@ -131,6 +182,9 @@
     <t>Malnad College of Engineering</t>
   </si>
   <si>
+    <t>4MC</t>
+  </si>
+  <si>
     <t>Hassan</t>
   </si>
   <si>
@@ -140,6 +194,9 @@
     <t>JSS Science and Technology University</t>
   </si>
   <si>
+    <t>4JS</t>
+  </si>
+  <si>
     <t>Mysuru</t>
   </si>
   <si>
@@ -149,12 +206,18 @@
     <t>NIE Institute of Technology</t>
   </si>
   <si>
+    <t>4NI</t>
+  </si>
+  <si>
     <t>Koorgalli, Hootagalli, Mysuru 570018</t>
   </si>
   <si>
     <t>Channabasaveshwara Institute of Technology</t>
   </si>
   <si>
+    <t>1CT</t>
+  </si>
+  <si>
     <t>NH 206, Gubbi, Tumakuru 572216</t>
   </si>
   <si>
@@ -176,16 +239,16 @@
     <t>Filling in your own list</t>
   </si>
   <si>
-    <t>•  Keep the three column headings on row 1 exactly as they are: College Name, Location, Address.</t>
-  </si>
-  <si>
-    <t>•  Only College Name is required. Location and Address may be left blank.</t>
+    <t>•  Keep the column headings on row 1: College Name, College Code, Location, Address.</t>
+  </si>
+  <si>
+    <t>•  Only College Name is required. Code, Location and Address may be left blank.</t>
   </si>
   <si>
     <t>•  One college per row. Do not merge cells or leave blank rows in the middle.</t>
   </si>
   <si>
-    <t>•  Names are saved in CAPITALS automatically — type them however you like.</t>
+    <t>•  Names and codes are saved in CAPITALS automatically — type them however you like.</t>
   </si>
   <si>
     <t>•  The list is sorted alphabetically by the portal, so the order here does not matter.</t>
@@ -200,10 +263,10 @@
     <t>•  The importer reads the headings, so the columns can be in any order.</t>
   </si>
   <si>
-    <t>•  If row 1 has no recognisable headings, the first three columns are read as</t>
-  </si>
-  <si>
-    <t>•  College Name, Location and Address in that order.</t>
+    <t>•  If row 1 has no recognisable headings, the first four columns are read as</t>
+  </si>
+  <si>
+    <t>•  College Name, College Code, Location and Address in that order.</t>
   </si>
 </sst>
 </file>
@@ -643,15 +706,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="46" customWidth="1"/>
-    <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="3" max="3" width="62" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="62" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -661,229 +725,292 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" ht="19" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" ht="19" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" ht="19" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" ht="19" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" ht="19" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" ht="19" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" ht="19" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" ht="19" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="6" ht="19" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" ht="19" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="7" ht="19" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7" ht="19" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="8" ht="19" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" ht="19" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="9" ht="19" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" ht="19" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>4</v>
+        <v>27</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="10" ht="19" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="10" ht="19" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>4</v>
+        <v>30</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="11" ht="19" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="11" ht="19" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>4</v>
+        <v>33</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="12" ht="19" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="12" ht="19" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>4</v>
+        <v>36</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="13" ht="19" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="13" ht="19" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>4</v>
+        <v>39</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="14" ht="19" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="14" ht="19" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>4</v>
+        <v>42</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="15" ht="19" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="15" ht="19" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>4</v>
+        <v>45</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="16" ht="19" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="16" ht="19" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>32</v>
+        <v>47</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>33</v>
+        <v>48</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="17" ht="19" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>49</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="17" ht="19" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="18" ht="19" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>53</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="18" ht="19" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>38</v>
+        <v>55</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>39</v>
+        <v>56</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="19" ht="19" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>57</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="19" ht="19" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>41</v>
+        <v>59</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>42</v>
+        <v>60</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="20" ht="19" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>61</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="20" ht="19" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>44</v>
+        <v>63</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>42</v>
+        <v>64</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="21" ht="19" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>61</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="21" ht="19" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>46</v>
+        <v>66</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>33</v>
+        <v>67</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>47</v>
+        <v>49</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>68</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C21"/>
+  <autoFilter ref="A1:D21"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -900,162 +1027,162 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>48</v>
+        <v>69</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>49</v>
+        <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>48</v>
+        <v>69</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>48</v>
+        <v>69</v>
       </c>
     </row>
     <row r="3" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>48</v>
+        <v>69</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>50</v>
+        <v>71</v>
       </c>
     </row>
     <row r="4" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>48</v>
+        <v>69</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>51</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>48</v>
+        <v>69</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>52</v>
+        <v>73</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>48</v>
+        <v>69</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>48</v>
+        <v>69</v>
       </c>
     </row>
     <row r="7" ht="26" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>48</v>
+        <v>69</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>53</v>
+        <v>74</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>48</v>
+        <v>69</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>48</v>
+        <v>69</v>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>48</v>
+        <v>69</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>54</v>
+        <v>75</v>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>48</v>
+        <v>69</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>55</v>
+        <v>76</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>48</v>
+        <v>69</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>56</v>
+        <v>77</v>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>48</v>
+        <v>69</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>57</v>
+        <v>78</v>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>48</v>
+        <v>69</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>58</v>
+        <v>79</v>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>48</v>
+        <v>69</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>59</v>
+        <v>80</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>48</v>
+        <v>69</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>48</v>
+        <v>69</v>
       </c>
     </row>
     <row r="16" ht="26" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>48</v>
+        <v>69</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>60</v>
+        <v>81</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>48</v>
+        <v>69</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>48</v>
+        <v>69</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>48</v>
+        <v>69</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>61</v>
+        <v>82</v>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>48</v>
+        <v>69</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>62</v>
+        <v>83</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>48</v>
+        <v>69</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>63</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>

</xml_diff>